<commit_message>
Complete task12 multi-product commit handoff
</commit_message>
<xml_diff>
--- a/data/samples/price_rules.xlsx
+++ b/data/samples/price_rules.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,9 +529,10 @@
           <t>round</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -539,6 +540,7 @@
           <t>10</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -697,7 +699,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -710,7 +712,6 @@
           <t>none</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>True</t>
@@ -721,7 +722,120 @@
           <t>13</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PRICE-B-0-1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>全平台B级加价0.1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>fixed_markup</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PRICE-0-1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>蚂蚁加价0.1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fixed_markup</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>